<commit_message>
bieu mau van hanh luyen coc
</commit_message>
<xml_diff>
--- a/VanHanhCD1/wwwroot/templates/BMVH_LoDOLOMIT2.xlsx
+++ b/VanHanhCD1/wwwroot/templates/BMVH_LoDOLOMIT2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03. Project Hoa Phat\07. Backend\VanHanhCD1_API-main\VanHanhCD1\wwwroot\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\02. Du An Hoa Phat\API\VanHanhCD1_API-release\VanHanhCD1\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E048988-8D08-4BD7-A5F8-6E7EDF3841B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783F7213-B883-4D0D-A101-D32C2103E947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="578" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="578" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -18,10 +18,19 @@
     <sheet name="Ca Ngay" sheetId="3" r:id="rId3"/>
     <sheet name="Ca Dem" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -23558,6 +23567,88 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <WorkflowStatus xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">Soạn thảo</WorkflowStatus>
+    <WorkflowURL xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">&lt;a href='/workflow/SitePages/Workflow.aspx?mode=2&amp;LID=254ea173-42a4-4b32-afbf-3bf770118a86&amp;itemID=133721' target='_blank'&gt;OS2312121972&lt;/a&gt;</WorkflowURL>
+    <DocumentCategoryData xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
+    <DocumentCategoryID xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">161</DocumentCategoryID>
+    <Abstract xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
+    <WorkflowID xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">132</WorkflowID>
+    <Index xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
+    <DocumentCategory xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">161;#Tài liệu tham khảo</DocumentCategory>
+    <Required xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
+    <RequestCode xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">OS2312121972</RequestCode>
+    <Workflow xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">Quy trình Trình ký online</Workflow>
+    <_dlc_DocId xmlns="998bb92a-6464-419f-a0f9-924a868214cd">DQURWQRM4CD3-1578625852-569709</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="998bb92a-6464-419f-a0f9-924a868214cd">
+      <Url>https://eoffice.hoaphat.com.vn/record23/dungquat/_layouts/15/DocIdRedir.aspx?ID=DQURWQRM4CD3-1578625852-569709</Url>
+      <Description>DQURWQRM4CD3-1578625852-569709</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004E80E4044EF8C64283904840BF522E83" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0cd73694a5f7c96a9bd28f75f6889f88">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="998bb92a-6464-419f-a0f9-924a868214cd" xmlns:ns3="0861895e-72d3-49e1-9fd6-30e326ecfd33" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d17a98453237ee78ca208d86170a4f1" ns2:_="" ns3:_="">
     <xsd:import namespace="998bb92a-6464-419f-a0f9-924a868214cd"/>
@@ -23807,89 +23898,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6FEED28-00EE-4310-9380-BC6DE9840F9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B898D909-4CB7-4B8E-BF6A-C53B57E30FF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <WorkflowStatus xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">Soạn thảo</WorkflowStatus>
-    <WorkflowURL xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">&lt;a href='/workflow/SitePages/Workflow.aspx?mode=2&amp;LID=254ea173-42a4-4b32-afbf-3bf770118a86&amp;itemID=133721' target='_blank'&gt;OS2312121972&lt;/a&gt;</WorkflowURL>
-    <DocumentCategoryData xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
-    <DocumentCategoryID xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">161</DocumentCategoryID>
-    <Abstract xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
-    <WorkflowID xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">132</WorkflowID>
-    <Index xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
-    <DocumentCategory xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">161;#Tài liệu tham khảo</DocumentCategory>
-    <Required xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33" xsi:nil="true"/>
-    <RequestCode xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">OS2312121972</RequestCode>
-    <Workflow xmlns="0861895e-72d3-49e1-9fd6-30e326ecfd33">Quy trình Trình ký online</Workflow>
-    <_dlc_DocId xmlns="998bb92a-6464-419f-a0f9-924a868214cd">DQURWQRM4CD3-1578625852-569709</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="998bb92a-6464-419f-a0f9-924a868214cd">
-      <Url>https://eoffice.hoaphat.com.vn/record23/dungquat/_layouts/15/DocIdRedir.aspx?ID=DQURWQRM4CD3-1578625852-569709</Url>
-      <Description>DQURWQRM4CD3-1578625852-569709</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{352342B9-2286-4254-A508-C505873421E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0861895e-72d3-49e1-9fd6-30e326ecfd33"/>
+    <ds:schemaRef ds:uri="998bb92a-6464-419f-a0f9-924a868214cd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FA947CA-8091-45E6-8549-EEAFAB5613C9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23906,31 +23942,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6FEED28-00EE-4310-9380-BC6DE9840F9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B898D909-4CB7-4B8E-BF6A-C53B57E30FF4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{352342B9-2286-4254-A508-C505873421E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0861895e-72d3-49e1-9fd6-30e326ecfd33"/>
-    <ds:schemaRef ds:uri="998bb92a-6464-419f-a0f9-924a868214cd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>